<commit_message>
Created tables in SQL
</commit_message>
<xml_diff>
--- a/data/raw/synthetic_tiktok_shop_sales_2024_DOMINANT.xlsx
+++ b/data/raw/synthetic_tiktok_shop_sales_2024_DOMINANT.xlsx
@@ -1,36 +1,52 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\defaultuser0\Documents\nicosys-portfolio-ecom\data\raw\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E63CD1A2-A34A-4EAF-A825-E9907347D5E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="2652" yWindow="2652" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TikTok_Sales" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="TikTok_Sales" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+  <si>
+    <t>total_sales</t>
+  </si>
+  <si>
+    <t>order_date</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -49,81 +65,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -411,2416 +368,2411 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B300"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>date</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>total_sales</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="n">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="1">
         <v>45292</v>
       </c>
-      <c r="B2" t="n">
+      <c r="B2">
         <v>2996.84</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="1" t="n">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="1">
         <v>45293</v>
       </c>
-      <c r="B3" t="n">
+      <c r="B3">
         <v>3167.73</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="1" t="n">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
         <v>45294</v>
       </c>
-      <c r="B4" t="n">
+      <c r="B4">
         <v>4251.54</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="1" t="n">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
         <v>45295</v>
       </c>
-      <c r="B5" t="n">
-        <v>4285.11</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="B5">
+        <v>4285.1099999999997</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
         <v>45297</v>
       </c>
-      <c r="B6" t="n">
+      <c r="B6">
         <v>2033.86</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="1" t="n">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
         <v>45298</v>
       </c>
-      <c r="B7" t="n">
-        <v>2093.47</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="B7">
+        <v>2093.4699999999998</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
         <v>45299</v>
       </c>
-      <c r="B8" t="n">
+      <c r="B8">
         <v>3598.2</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="1" t="n">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" s="1">
         <v>45300</v>
       </c>
-      <c r="B9" t="n">
+      <c r="B9">
         <v>3947.81</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="1" t="n">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" s="1">
         <v>45301</v>
       </c>
-      <c r="B10" t="n">
+      <c r="B10">
         <v>3152.51</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="1" t="n">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" s="1">
         <v>45302</v>
       </c>
-      <c r="B11" t="n">
+      <c r="B11">
         <v>2682.16</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="1" t="n">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" s="1">
         <v>45303</v>
       </c>
-      <c r="B12" t="n">
+      <c r="B12">
         <v>4437.29</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="1" t="n">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" s="1">
         <v>45304</v>
       </c>
-      <c r="B13" t="n">
+      <c r="B13">
         <v>3017.82</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="1" t="n">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" s="1">
         <v>45305</v>
       </c>
-      <c r="B14" t="n">
-        <v>4764.9</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="n">
+      <c r="B14">
+        <v>4764.8999999999996</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" s="1">
         <v>45306</v>
       </c>
-      <c r="B15" t="n">
+      <c r="B15">
         <v>3733.33</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="1" t="n">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" s="1">
         <v>45307</v>
       </c>
-      <c r="B16" t="n">
+      <c r="B16">
         <v>1853.12</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="1" t="n">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" s="1">
         <v>45308</v>
       </c>
-      <c r="B17" t="n">
+      <c r="B17">
         <v>4921.93</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="1" t="n">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" s="1">
         <v>45309</v>
       </c>
-      <c r="B18" t="n">
+      <c r="B18">
         <v>3895.5</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="1" t="n">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" s="1">
         <v>45310</v>
       </c>
-      <c r="B19" t="n">
+      <c r="B19">
         <v>3737.38</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="1" t="n">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" s="1">
         <v>45312</v>
       </c>
-      <c r="B20" t="n">
+      <c r="B20">
         <v>4316.08</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="1" t="n">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" s="1">
         <v>45315</v>
       </c>
-      <c r="B21" t="n">
+      <c r="B21">
         <v>4786.76</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="1" t="n">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" s="1">
         <v>45316</v>
       </c>
-      <c r="B22" t="n">
+      <c r="B22">
         <v>3131.1</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="1" t="n">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" s="1">
         <v>45317</v>
       </c>
-      <c r="B23" t="n">
+      <c r="B23">
         <v>4220.62</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="1" t="n">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24" s="1">
         <v>45319</v>
       </c>
-      <c r="B24" t="n">
+      <c r="B24">
         <v>1614.82</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="1" t="n">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A25" s="1">
         <v>45320</v>
       </c>
-      <c r="B25" t="n">
+      <c r="B25">
         <v>3808.32</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="1" t="n">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26" s="1">
         <v>45321</v>
       </c>
-      <c r="B26" t="n">
+      <c r="B26">
         <v>2992.47</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="1" t="n">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A27" s="1">
         <v>45322</v>
       </c>
-      <c r="B27" t="n">
+      <c r="B27">
         <v>4541.58</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="1" t="n">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A28" s="1">
         <v>45324</v>
       </c>
-      <c r="B28" t="n">
-        <v>2336.93</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="1" t="n">
+      <c r="B28">
+        <v>2336.9299999999998</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A29" s="1">
         <v>45325</v>
       </c>
-      <c r="B29" t="n">
-        <v>4211.56</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="1" t="n">
+      <c r="B29">
+        <v>4211.5600000000004</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A30" s="1">
         <v>45326</v>
       </c>
-      <c r="B30" t="n">
-        <v>4432.52</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="1" t="n">
+      <c r="B30">
+        <v>4432.5200000000004</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A31" s="1">
         <v>45327</v>
       </c>
-      <c r="B31" t="n">
+      <c r="B31">
         <v>2803.95</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="1" t="n">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A32" s="1">
         <v>45328</v>
       </c>
-      <c r="B32" t="n">
-        <v>4751.39</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="1" t="n">
+      <c r="B32">
+        <v>4751.3900000000003</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A33" s="1">
         <v>45330</v>
       </c>
-      <c r="B33" t="n">
+      <c r="B33">
         <v>1934.11</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="1" t="n">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A34" s="1">
         <v>45331</v>
       </c>
-      <c r="B34" t="n">
+      <c r="B34">
         <v>1959.72</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="1" t="n">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A35" s="1">
         <v>45332</v>
       </c>
-      <c r="B35" t="n">
-        <v>2533.78</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="1" t="n">
+      <c r="B35">
+        <v>2533.7800000000002</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A36" s="1">
         <v>45335</v>
       </c>
-      <c r="B36" t="n">
-        <v>4677.23</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="1" t="n">
+      <c r="B36">
+        <v>4677.2299999999996</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A37" s="1">
         <v>45336</v>
       </c>
-      <c r="B37" t="n">
+      <c r="B37">
         <v>3090.24</v>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="1" t="n">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A38" s="1">
         <v>45337</v>
       </c>
-      <c r="B38" t="n">
+      <c r="B38">
         <v>3977.88</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="1" t="n">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A39" s="1">
         <v>45338</v>
       </c>
-      <c r="B39" t="n">
+      <c r="B39">
         <v>2710.23</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="1" t="n">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A40" s="1">
         <v>45339</v>
       </c>
-      <c r="B40" t="n">
+      <c r="B40">
         <v>1598.82</v>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="1" t="n">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A41" s="1">
         <v>45340</v>
       </c>
-      <c r="B41" t="n">
+      <c r="B41">
         <v>2396.37</v>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="1" t="n">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A42" s="1">
         <v>45341</v>
       </c>
-      <c r="B42" t="n">
+      <c r="B42">
         <v>2185.13</v>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="1" t="n">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A43" s="1">
         <v>45342</v>
       </c>
-      <c r="B43" t="n">
+      <c r="B43">
         <v>3023.87</v>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="1" t="n">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A44" s="1">
         <v>45343</v>
       </c>
-      <c r="B44" t="n">
+      <c r="B44">
         <v>1685.95</v>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="1" t="n">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A45" s="1">
         <v>45345</v>
       </c>
-      <c r="B45" t="n">
+      <c r="B45">
         <v>3363.79</v>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="1" t="n">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A46" s="1">
         <v>45346</v>
       </c>
-      <c r="B46" t="n">
+      <c r="B46">
         <v>3548.91</v>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="1" t="n">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A47" s="1">
         <v>45347</v>
       </c>
-      <c r="B47" t="n">
+      <c r="B47">
         <v>1711.83</v>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="1" t="n">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A48" s="1">
         <v>45348</v>
       </c>
-      <c r="B48" t="n">
+      <c r="B48">
         <v>1874.24</v>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="1" t="n">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A49" s="1">
         <v>45349</v>
       </c>
-      <c r="B49" t="n">
+      <c r="B49">
         <v>4609.28</v>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="1" t="n">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A50" s="1">
         <v>45351</v>
       </c>
-      <c r="B50" t="n">
+      <c r="B50">
         <v>4242.53</v>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="1" t="n">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A51" s="1">
         <v>45353</v>
       </c>
-      <c r="B51" t="n">
-        <v>4326.94</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="1" t="n">
+      <c r="B51">
+        <v>4326.9399999999996</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A52" s="1">
         <v>45354</v>
       </c>
-      <c r="B52" t="n">
+      <c r="B52">
         <v>4320.29</v>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="1" t="n">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A53" s="1">
         <v>45355</v>
       </c>
-      <c r="B53" t="n">
+      <c r="B53">
         <v>4003.28</v>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="1" t="n">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A54" s="1">
         <v>45356</v>
       </c>
-      <c r="B54" t="n">
+      <c r="B54">
         <v>3106.44</v>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="1" t="n">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A55" s="1">
         <v>45357</v>
       </c>
-      <c r="B55" t="n">
+      <c r="B55">
         <v>2259.21</v>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="1" t="n">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A56" s="1">
         <v>45358</v>
       </c>
-      <c r="B56" t="n">
+      <c r="B56">
         <v>3295.37</v>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="1" t="n">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A57" s="1">
         <v>45359</v>
       </c>
-      <c r="B57" t="n">
+      <c r="B57">
         <v>1802.1</v>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="1" t="n">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A58" s="1">
         <v>45360</v>
       </c>
-      <c r="B58" t="n">
+      <c r="B58">
         <v>3216.71</v>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="1" t="n">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A59" s="1">
         <v>45361</v>
       </c>
-      <c r="B59" t="n">
+      <c r="B59">
         <v>2889.2</v>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="1" t="n">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A60" s="1">
         <v>45362</v>
       </c>
-      <c r="B60" t="n">
+      <c r="B60">
         <v>2296.71</v>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="1" t="n">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A61" s="1">
         <v>45363</v>
       </c>
-      <c r="B61" t="n">
+      <c r="B61">
         <v>2645.06</v>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="1" t="n">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A62" s="1">
         <v>45364</v>
       </c>
-      <c r="B62" t="n">
+      <c r="B62">
         <v>4633.95</v>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="1" t="n">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A63" s="1">
         <v>45365</v>
       </c>
-      <c r="B63" t="n">
+      <c r="B63">
         <v>3844.91</v>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="1" t="n">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A64" s="1">
         <v>45366</v>
       </c>
-      <c r="B64" t="n">
-        <v>2423.05</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="1" t="n">
+      <c r="B64">
+        <v>2423.0500000000002</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A65" s="1">
         <v>45367</v>
       </c>
-      <c r="B65" t="n">
+      <c r="B65">
         <v>4012.13</v>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="1" t="n">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A66" s="1">
         <v>45368</v>
       </c>
-      <c r="B66" t="n">
+      <c r="B66">
         <v>3491.43</v>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="1" t="n">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A67" s="1">
         <v>45369</v>
       </c>
-      <c r="B67" t="n">
+      <c r="B67">
         <v>4999.76</v>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="1" t="n">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A68" s="1">
         <v>45370</v>
       </c>
-      <c r="B68" t="n">
+      <c r="B68">
         <v>1829.55</v>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="1" t="n">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A69" s="1">
         <v>45371</v>
       </c>
-      <c r="B69" t="n">
+      <c r="B69">
         <v>3814.31</v>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="1" t="n">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A70" s="1">
         <v>45372</v>
       </c>
-      <c r="B70" t="n">
+      <c r="B70">
         <v>2769.64</v>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="1" t="n">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A71" s="1">
         <v>45373</v>
       </c>
-      <c r="B71" t="n">
+      <c r="B71">
         <v>4702.13</v>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="1" t="n">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A72" s="1">
         <v>45375</v>
       </c>
-      <c r="B72" t="n">
+      <c r="B72">
         <v>4570.66</v>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" s="1" t="n">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A73" s="1">
         <v>45376</v>
       </c>
-      <c r="B73" t="n">
+      <c r="B73">
         <v>2217.08</v>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="1" t="n">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A74" s="1">
         <v>45378</v>
       </c>
-      <c r="B74" t="n">
+      <c r="B74">
         <v>4240.07</v>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="1" t="n">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A75" s="1">
         <v>45379</v>
       </c>
-      <c r="B75" t="n">
+      <c r="B75">
         <v>3039.79</v>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" s="1" t="n">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A76" s="1">
         <v>45380</v>
       </c>
-      <c r="B76" t="n">
+      <c r="B76">
         <v>2179.21</v>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" s="1" t="n">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A77" s="1">
         <v>45381</v>
       </c>
-      <c r="B77" t="n">
+      <c r="B77">
         <v>3772.5</v>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" s="1" t="n">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A78" s="1">
         <v>45382</v>
       </c>
-      <c r="B78" t="n">
+      <c r="B78">
         <v>2713.26</v>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" s="1" t="n">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A79" s="1">
         <v>45383</v>
       </c>
-      <c r="B79" t="n">
+      <c r="B79">
         <v>3808.37</v>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" s="1" t="n">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A80" s="1">
         <v>45384</v>
       </c>
-      <c r="B80" t="n">
-        <v>2429.8</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="1" t="n">
+      <c r="B80">
+        <v>2429.8000000000002</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A81" s="1">
         <v>45385</v>
       </c>
-      <c r="B81" t="n">
+      <c r="B81">
         <v>3991.76</v>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" s="1" t="n">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A82" s="1">
         <v>45386</v>
       </c>
-      <c r="B82" t="n">
+      <c r="B82">
         <v>1689.57</v>
       </c>
     </row>
-    <row r="83">
-      <c r="A83" s="1" t="n">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A83" s="1">
         <v>45387</v>
       </c>
-      <c r="B83" t="n">
+      <c r="B83">
         <v>4681.78</v>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" s="1" t="n">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A84" s="1">
         <v>45388</v>
       </c>
-      <c r="B84" t="n">
+      <c r="B84">
         <v>4044.41</v>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" s="1" t="n">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A85" s="1">
         <v>45390</v>
       </c>
-      <c r="B85" t="n">
-        <v>2574.57</v>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="1" t="n">
+      <c r="B85">
+        <v>2574.5700000000002</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A86" s="1">
         <v>45392</v>
       </c>
-      <c r="B86" t="n">
+      <c r="B86">
         <v>2940.34</v>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" s="1" t="n">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A87" s="1">
         <v>45393</v>
       </c>
-      <c r="B87" t="n">
+      <c r="B87">
         <v>4598.83</v>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" s="1" t="n">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A88" s="1">
         <v>45394</v>
       </c>
-      <c r="B88" t="n">
+      <c r="B88">
         <v>1794.37</v>
       </c>
     </row>
-    <row r="89">
-      <c r="A89" s="1" t="n">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A89" s="1">
         <v>45396</v>
       </c>
-      <c r="B89" t="n">
+      <c r="B89">
         <v>4558.63</v>
       </c>
     </row>
-    <row r="90">
-      <c r="A90" s="1" t="n">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A90" s="1">
         <v>45397</v>
       </c>
-      <c r="B90" t="n">
+      <c r="B90">
         <v>2230.12</v>
       </c>
     </row>
-    <row r="91">
-      <c r="A91" s="1" t="n">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A91" s="1">
         <v>45398</v>
       </c>
-      <c r="B91" t="n">
+      <c r="B91">
         <v>1618</v>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" s="1" t="n">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A92" s="1">
         <v>45399</v>
       </c>
-      <c r="B92" t="n">
-        <v>4113.02</v>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="1" t="n">
+      <c r="B92">
+        <v>4113.0200000000004</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A93" s="1">
         <v>45400</v>
       </c>
-      <c r="B93" t="n">
+      <c r="B93">
         <v>4062.92</v>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" s="1" t="n">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A94" s="1">
         <v>45401</v>
       </c>
-      <c r="B94" t="n">
+      <c r="B94">
         <v>3352.69</v>
       </c>
     </row>
-    <row r="95">
-      <c r="A95" s="1" t="n">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A95" s="1">
         <v>45402</v>
       </c>
-      <c r="B95" t="n">
+      <c r="B95">
         <v>2019.24</v>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" s="1" t="n">
+    <row r="96" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A96" s="1">
         <v>45403</v>
       </c>
-      <c r="B96" t="n">
+      <c r="B96">
         <v>2200.79</v>
       </c>
     </row>
-    <row r="97">
-      <c r="A97" s="1" t="n">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A97" s="1">
         <v>45405</v>
       </c>
-      <c r="B97" t="n">
+      <c r="B97">
         <v>3383.46</v>
       </c>
     </row>
-    <row r="98">
-      <c r="A98" s="1" t="n">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A98" s="1">
         <v>45406</v>
       </c>
-      <c r="B98" t="n">
+      <c r="B98">
         <v>2364.98</v>
       </c>
     </row>
-    <row r="99">
-      <c r="A99" s="1" t="n">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A99" s="1">
         <v>45407</v>
       </c>
-      <c r="B99" t="n">
+      <c r="B99">
         <v>3996.67</v>
       </c>
     </row>
-    <row r="100">
-      <c r="A100" s="1" t="n">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A100" s="1">
         <v>45408</v>
       </c>
-      <c r="B100" t="n">
+      <c r="B100">
         <v>1907.27</v>
       </c>
     </row>
-    <row r="101">
-      <c r="A101" s="1" t="n">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A101" s="1">
         <v>45409</v>
       </c>
-      <c r="B101" t="n">
+      <c r="B101">
         <v>3679.25</v>
       </c>
     </row>
-    <row r="102">
-      <c r="A102" s="1" t="n">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A102" s="1">
         <v>45410</v>
       </c>
-      <c r="B102" t="n">
+      <c r="B102">
         <v>4920.47</v>
       </c>
     </row>
-    <row r="103">
-      <c r="A103" s="1" t="n">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A103" s="1">
         <v>45411</v>
       </c>
-      <c r="B103" t="n">
+      <c r="B103">
         <v>2090.38</v>
       </c>
     </row>
-    <row r="104">
-      <c r="A104" s="1" t="n">
+    <row r="104" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A104" s="1">
         <v>45412</v>
       </c>
-      <c r="B104" t="n">
+      <c r="B104">
         <v>2029.26</v>
       </c>
     </row>
-    <row r="105">
-      <c r="A105" s="1" t="n">
+    <row r="105" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A105" s="1">
         <v>45413</v>
       </c>
-      <c r="B105" t="n">
+      <c r="B105">
         <v>2223.23</v>
       </c>
     </row>
-    <row r="106">
-      <c r="A106" s="1" t="n">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A106" s="1">
         <v>45414</v>
       </c>
-      <c r="B106" t="n">
+      <c r="B106">
         <v>2438.61</v>
       </c>
     </row>
-    <row r="107">
-      <c r="A107" s="1" t="n">
+    <row r="107" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A107" s="1">
         <v>45415</v>
       </c>
-      <c r="B107" t="n">
+      <c r="B107">
         <v>1915.9</v>
       </c>
     </row>
-    <row r="108">
-      <c r="A108" s="1" t="n">
+    <row r="108" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A108" s="1">
         <v>45416</v>
       </c>
-      <c r="B108" t="n">
+      <c r="B108">
         <v>3689.79</v>
       </c>
     </row>
-    <row r="109">
-      <c r="A109" s="1" t="n">
+    <row r="109" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A109" s="1">
         <v>45417</v>
       </c>
-      <c r="B109" t="n">
-        <v>2448.68</v>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" s="1" t="n">
+      <c r="B109">
+        <v>2448.6799999999998</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A110" s="1">
         <v>45419</v>
       </c>
-      <c r="B110" t="n">
+      <c r="B110">
         <v>3776.13</v>
       </c>
     </row>
-    <row r="111">
-      <c r="A111" s="1" t="n">
+    <row r="111" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A111" s="1">
         <v>45420</v>
       </c>
-      <c r="B111" t="n">
+      <c r="B111">
         <v>3307.33</v>
       </c>
     </row>
-    <row r="112">
-      <c r="A112" s="1" t="n">
+    <row r="112" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A112" s="1">
         <v>45421</v>
       </c>
-      <c r="B112" t="n">
+      <c r="B112">
         <v>1783.05</v>
       </c>
     </row>
-    <row r="113">
-      <c r="A113" s="1" t="n">
+    <row r="113" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A113" s="1">
         <v>45422</v>
       </c>
-      <c r="B113" t="n">
+      <c r="B113">
         <v>1857.21</v>
       </c>
     </row>
-    <row r="114">
-      <c r="A114" s="1" t="n">
+    <row r="114" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A114" s="1">
         <v>45423</v>
       </c>
-      <c r="B114" t="n">
+      <c r="B114">
         <v>4641.54</v>
       </c>
     </row>
-    <row r="115">
-      <c r="A115" s="1" t="n">
+    <row r="115" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A115" s="1">
         <v>45425</v>
       </c>
-      <c r="B115" t="n">
+      <c r="B115">
         <v>1576.97</v>
       </c>
     </row>
-    <row r="116">
-      <c r="A116" s="1" t="n">
+    <row r="116" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A116" s="1">
         <v>45426</v>
       </c>
-      <c r="B116" t="n">
+      <c r="B116">
         <v>2339.33</v>
       </c>
     </row>
-    <row r="117">
-      <c r="A117" s="1" t="n">
+    <row r="117" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A117" s="1">
         <v>45427</v>
       </c>
-      <c r="B117" t="n">
+      <c r="B117">
         <v>2313.38</v>
       </c>
     </row>
-    <row r="118">
-      <c r="A118" s="1" t="n">
+    <row r="118" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A118" s="1">
         <v>45428</v>
       </c>
-      <c r="B118" t="n">
+      <c r="B118">
         <v>3177.33</v>
       </c>
     </row>
-    <row r="119">
-      <c r="A119" s="1" t="n">
+    <row r="119" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A119" s="1">
         <v>45430</v>
       </c>
-      <c r="B119" t="n">
-        <v>2048.97</v>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" s="1" t="n">
+      <c r="B119">
+        <v>2048.9699999999998</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A120" s="1">
         <v>45431</v>
       </c>
-      <c r="B120" t="n">
+      <c r="B120">
         <v>1691.65</v>
       </c>
     </row>
-    <row r="121">
-      <c r="A121" s="1" t="n">
+    <row r="121" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A121" s="1">
         <v>45433</v>
       </c>
-      <c r="B121" t="n">
+      <c r="B121">
         <v>3133.57</v>
       </c>
     </row>
-    <row r="122">
-      <c r="A122" s="1" t="n">
+    <row r="122" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A122" s="1">
         <v>45434</v>
       </c>
-      <c r="B122" t="n">
+      <c r="B122">
         <v>3677.2</v>
       </c>
     </row>
-    <row r="123">
-      <c r="A123" s="1" t="n">
+    <row r="123" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A123" s="1">
         <v>45436</v>
       </c>
-      <c r="B123" t="n">
+      <c r="B123">
         <v>2038.02</v>
       </c>
     </row>
-    <row r="124">
-      <c r="A124" s="1" t="n">
+    <row r="124" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A124" s="1">
         <v>45437</v>
       </c>
-      <c r="B124" t="n">
+      <c r="B124">
         <v>1979.86</v>
       </c>
     </row>
-    <row r="125">
-      <c r="A125" s="1" t="n">
+    <row r="125" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A125" s="1">
         <v>45438</v>
       </c>
-      <c r="B125" t="n">
+      <c r="B125">
         <v>3709.85</v>
       </c>
     </row>
-    <row r="126">
-      <c r="A126" s="1" t="n">
+    <row r="126" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A126" s="1">
         <v>45439</v>
       </c>
-      <c r="B126" t="n">
+      <c r="B126">
         <v>2393.29</v>
       </c>
     </row>
-    <row r="127">
-      <c r="A127" s="1" t="n">
+    <row r="127" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A127" s="1">
         <v>45440</v>
       </c>
-      <c r="B127" t="n">
-        <v>4519.52</v>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" s="1" t="n">
+      <c r="B127">
+        <v>4519.5200000000004</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A128" s="1">
         <v>45441</v>
       </c>
-      <c r="B128" t="n">
+      <c r="B128">
         <v>4734.79</v>
       </c>
     </row>
-    <row r="129">
-      <c r="A129" s="1" t="n">
+    <row r="129" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A129" s="1">
         <v>45442</v>
       </c>
-      <c r="B129" t="n">
+      <c r="B129">
         <v>4003.51</v>
       </c>
     </row>
-    <row r="130">
-      <c r="A130" s="1" t="n">
+    <row r="130" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A130" s="1">
         <v>45443</v>
       </c>
-      <c r="B130" t="n">
+      <c r="B130">
         <v>1763.3</v>
       </c>
     </row>
-    <row r="131">
-      <c r="A131" s="1" t="n">
+    <row r="131" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A131" s="1">
         <v>45444</v>
       </c>
-      <c r="B131" t="n">
+      <c r="B131">
         <v>1602.64</v>
       </c>
     </row>
-    <row r="132">
-      <c r="A132" s="1" t="n">
+    <row r="132" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A132" s="1">
         <v>45445</v>
       </c>
-      <c r="B132" t="n">
+      <c r="B132">
         <v>1898</v>
       </c>
     </row>
-    <row r="133">
-      <c r="A133" s="1" t="n">
+    <row r="133" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A133" s="1">
         <v>45446</v>
       </c>
-      <c r="B133" t="n">
+      <c r="B133">
         <v>3453.88</v>
       </c>
     </row>
-    <row r="134">
-      <c r="A134" s="1" t="n">
+    <row r="134" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A134" s="1">
         <v>45448</v>
       </c>
-      <c r="B134" t="n">
+      <c r="B134">
         <v>2847.58</v>
       </c>
     </row>
-    <row r="135">
-      <c r="A135" s="1" t="n">
+    <row r="135" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A135" s="1">
         <v>45449</v>
       </c>
-      <c r="B135" t="n">
+      <c r="B135">
         <v>1915.42</v>
       </c>
     </row>
-    <row r="136">
-      <c r="A136" s="1" t="n">
+    <row r="136" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A136" s="1">
         <v>45450</v>
       </c>
-      <c r="B136" t="n">
+      <c r="B136">
         <v>1938.02</v>
       </c>
     </row>
-    <row r="137">
-      <c r="A137" s="1" t="n">
+    <row r="137" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A137" s="1">
         <v>45451</v>
       </c>
-      <c r="B137" t="n">
+      <c r="B137">
         <v>3392.44</v>
       </c>
     </row>
-    <row r="138">
-      <c r="A138" s="1" t="n">
+    <row r="138" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A138" s="1">
         <v>45452</v>
       </c>
-      <c r="B138" t="n">
+      <c r="B138">
         <v>4539.2</v>
       </c>
     </row>
-    <row r="139">
-      <c r="A139" s="1" t="n">
+    <row r="139" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A139" s="1">
         <v>45453</v>
       </c>
-      <c r="B139" t="n">
+      <c r="B139">
         <v>3164.19</v>
       </c>
     </row>
-    <row r="140">
-      <c r="A140" s="1" t="n">
+    <row r="140" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A140" s="1">
         <v>45454</v>
       </c>
-      <c r="B140" t="n">
+      <c r="B140">
         <v>3032.85</v>
       </c>
     </row>
-    <row r="141">
-      <c r="A141" s="1" t="n">
+    <row r="141" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A141" s="1">
         <v>45455</v>
       </c>
-      <c r="B141" t="n">
+      <c r="B141">
         <v>1549.2</v>
       </c>
     </row>
-    <row r="142">
-      <c r="A142" s="1" t="n">
+    <row r="142" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A142" s="1">
         <v>45456</v>
       </c>
-      <c r="B142" t="n">
+      <c r="B142">
         <v>3045.98</v>
       </c>
     </row>
-    <row r="143">
-      <c r="A143" s="1" t="n">
+    <row r="143" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A143" s="1">
         <v>45457</v>
       </c>
-      <c r="B143" t="n">
+      <c r="B143">
         <v>3274.31</v>
       </c>
     </row>
-    <row r="144">
-      <c r="A144" s="1" t="n">
+    <row r="144" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A144" s="1">
         <v>45459</v>
       </c>
-      <c r="B144" t="n">
+      <c r="B144">
         <v>2368.88</v>
       </c>
     </row>
-    <row r="145">
-      <c r="A145" s="1" t="n">
+    <row r="145" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A145" s="1">
         <v>45460</v>
       </c>
-      <c r="B145" t="n">
+      <c r="B145">
         <v>3220.48</v>
       </c>
     </row>
-    <row r="146">
-      <c r="A146" s="1" t="n">
+    <row r="146" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A146" s="1">
         <v>45461</v>
       </c>
-      <c r="B146" t="n">
-        <v>2092.03</v>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" s="1" t="n">
+      <c r="B146">
+        <v>2092.0300000000002</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A147" s="1">
         <v>45463</v>
       </c>
-      <c r="B147" t="n">
+      <c r="B147">
         <v>2247.92</v>
       </c>
     </row>
-    <row r="148">
-      <c r="A148" s="1" t="n">
+    <row r="148" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A148" s="1">
         <v>45464</v>
       </c>
-      <c r="B148" t="n">
+      <c r="B148">
         <v>2213.1</v>
       </c>
     </row>
-    <row r="149">
-      <c r="A149" s="1" t="n">
+    <row r="149" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A149" s="1">
         <v>45465</v>
       </c>
-      <c r="B149" t="n">
+      <c r="B149">
         <v>3587.92</v>
       </c>
     </row>
-    <row r="150">
-      <c r="A150" s="1" t="n">
+    <row r="150" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A150" s="1">
         <v>45466</v>
       </c>
-      <c r="B150" t="n">
+      <c r="B150">
         <v>4684.03</v>
       </c>
     </row>
-    <row r="151">
-      <c r="A151" s="1" t="n">
+    <row r="151" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A151" s="1">
         <v>45467</v>
       </c>
-      <c r="B151" t="n">
+      <c r="B151">
         <v>3293.33</v>
       </c>
     </row>
-    <row r="152">
-      <c r="A152" s="1" t="n">
+    <row r="152" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A152" s="1">
         <v>45468</v>
       </c>
-      <c r="B152" t="n">
+      <c r="B152">
         <v>2880.69</v>
       </c>
     </row>
-    <row r="153">
-      <c r="A153" s="1" t="n">
+    <row r="153" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A153" s="1">
         <v>45469</v>
       </c>
-      <c r="B153" t="n">
+      <c r="B153">
         <v>2937.46</v>
       </c>
     </row>
-    <row r="154">
-      <c r="A154" s="1" t="n">
+    <row r="154" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A154" s="1">
         <v>45470</v>
       </c>
-      <c r="B154" t="n">
-        <v>2103.43</v>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" s="1" t="n">
+      <c r="B154">
+        <v>2103.4299999999998</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A155" s="1">
         <v>45471</v>
       </c>
-      <c r="B155" t="n">
+      <c r="B155">
         <v>4224.09</v>
       </c>
     </row>
-    <row r="156">
-      <c r="A156" s="1" t="n">
+    <row r="156" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A156" s="1">
         <v>45472</v>
       </c>
-      <c r="B156" t="n">
+      <c r="B156">
         <v>2233.44</v>
       </c>
     </row>
-    <row r="157">
-      <c r="A157" s="1" t="n">
+    <row r="157" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A157" s="1">
         <v>45473</v>
       </c>
-      <c r="B157" t="n">
+      <c r="B157">
         <v>3931.92</v>
       </c>
     </row>
-    <row r="158">
-      <c r="A158" s="1" t="n">
+    <row r="158" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A158" s="1">
         <v>45475</v>
       </c>
-      <c r="B158" t="n">
+      <c r="B158">
         <v>4566.05</v>
       </c>
     </row>
-    <row r="159">
-      <c r="A159" s="1" t="n">
+    <row r="159" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A159" s="1">
         <v>45476</v>
       </c>
-      <c r="B159" t="n">
+      <c r="B159">
         <v>4054.01</v>
       </c>
     </row>
-    <row r="160">
-      <c r="A160" s="1" t="n">
+    <row r="160" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A160" s="1">
         <v>45478</v>
       </c>
-      <c r="B160" t="n">
+      <c r="B160">
         <v>3720.75</v>
       </c>
     </row>
-    <row r="161">
-      <c r="A161" s="1" t="n">
+    <row r="161" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A161" s="1">
         <v>45479</v>
       </c>
-      <c r="B161" t="n">
-        <v>4928.02</v>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" s="1" t="n">
+      <c r="B161">
+        <v>4928.0200000000004</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A162" s="1">
         <v>45480</v>
       </c>
-      <c r="B162" t="n">
-        <v>4970.48</v>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" s="1" t="n">
+      <c r="B162">
+        <v>4970.4799999999996</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A163" s="1">
         <v>45481</v>
       </c>
-      <c r="B163" t="n">
+      <c r="B163">
         <v>3872.44</v>
       </c>
     </row>
-    <row r="164">
-      <c r="A164" s="1" t="n">
+    <row r="164" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A164" s="1">
         <v>45482</v>
       </c>
-      <c r="B164" t="n">
-        <v>2145.01</v>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" s="1" t="n">
+      <c r="B164">
+        <v>2145.0100000000002</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A165" s="1">
         <v>45483</v>
       </c>
-      <c r="B165" t="n">
+      <c r="B165">
         <v>4827.41</v>
       </c>
     </row>
-    <row r="166">
-      <c r="A166" s="1" t="n">
+    <row r="166" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A166" s="1">
         <v>45484</v>
       </c>
-      <c r="B166" t="n">
+      <c r="B166">
         <v>2430.13</v>
       </c>
     </row>
-    <row r="167">
-      <c r="A167" s="1" t="n">
+    <row r="167" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A167" s="1">
         <v>45486</v>
       </c>
-      <c r="B167" t="n">
+      <c r="B167">
         <v>4710.47</v>
       </c>
     </row>
-    <row r="168">
-      <c r="A168" s="1" t="n">
+    <row r="168" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A168" s="1">
         <v>45488</v>
       </c>
-      <c r="B168" t="n">
+      <c r="B168">
         <v>3989.98</v>
       </c>
     </row>
-    <row r="169">
-      <c r="A169" s="1" t="n">
+    <row r="169" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A169" s="1">
         <v>45489</v>
       </c>
-      <c r="B169" t="n">
+      <c r="B169">
         <v>2006.91</v>
       </c>
     </row>
-    <row r="170">
-      <c r="A170" s="1" t="n">
+    <row r="170" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A170" s="1">
         <v>45490</v>
       </c>
-      <c r="B170" t="n">
-        <v>2553.24</v>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" s="1" t="n">
+      <c r="B170">
+        <v>2553.2399999999998</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A171" s="1">
         <v>45491</v>
       </c>
-      <c r="B171" t="n">
+      <c r="B171">
         <v>1894.93</v>
       </c>
     </row>
-    <row r="172">
-      <c r="A172" s="1" t="n">
+    <row r="172" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A172" s="1">
         <v>45492</v>
       </c>
-      <c r="B172" t="n">
+      <c r="B172">
         <v>3111.98</v>
       </c>
     </row>
-    <row r="173">
-      <c r="A173" s="1" t="n">
+    <row r="173" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A173" s="1">
         <v>45493</v>
       </c>
-      <c r="B173" t="n">
+      <c r="B173">
         <v>2501.1</v>
       </c>
     </row>
-    <row r="174">
-      <c r="A174" s="1" t="n">
+    <row r="174" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A174" s="1">
         <v>45494</v>
       </c>
-      <c r="B174" t="n">
+      <c r="B174">
         <v>3880.31</v>
       </c>
     </row>
-    <row r="175">
-      <c r="A175" s="1" t="n">
+    <row r="175" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A175" s="1">
         <v>45495</v>
       </c>
-      <c r="B175" t="n">
-        <v>2249.03</v>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" s="1" t="n">
+      <c r="B175">
+        <v>2249.0300000000002</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A176" s="1">
         <v>45496</v>
       </c>
-      <c r="B176" t="n">
+      <c r="B176">
         <v>2026.09</v>
       </c>
     </row>
-    <row r="177">
-      <c r="A177" s="1" t="n">
+    <row r="177" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A177" s="1">
         <v>45497</v>
       </c>
-      <c r="B177" t="n">
+      <c r="B177">
         <v>4187.84</v>
       </c>
     </row>
-    <row r="178">
-      <c r="A178" s="1" t="n">
+    <row r="178" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A178" s="1">
         <v>45498</v>
       </c>
-      <c r="B178" t="n">
+      <c r="B178">
         <v>4423.22</v>
       </c>
     </row>
-    <row r="179">
-      <c r="A179" s="1" t="n">
+    <row r="179" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A179" s="1">
         <v>45499</v>
       </c>
-      <c r="B179" t="n">
+      <c r="B179">
         <v>3312.84</v>
       </c>
     </row>
-    <row r="180">
-      <c r="A180" s="1" t="n">
+    <row r="180" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A180" s="1">
         <v>45500</v>
       </c>
-      <c r="B180" t="n">
+      <c r="B180">
         <v>3317.51</v>
       </c>
     </row>
-    <row r="181">
-      <c r="A181" s="1" t="n">
+    <row r="181" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A181" s="1">
         <v>45501</v>
       </c>
-      <c r="B181" t="n">
-        <v>2301.45</v>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" s="1" t="n">
+      <c r="B181">
+        <v>2301.4499999999998</v>
+      </c>
+    </row>
+    <row r="182" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A182" s="1">
         <v>45502</v>
       </c>
-      <c r="B182" t="n">
+      <c r="B182">
         <v>3061.74</v>
       </c>
     </row>
-    <row r="183">
-      <c r="A183" s="1" t="n">
+    <row r="183" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A183" s="1">
         <v>45503</v>
       </c>
-      <c r="B183" t="n">
+      <c r="B183">
         <v>1566.37</v>
       </c>
     </row>
-    <row r="184">
-      <c r="A184" s="1" t="n">
+    <row r="184" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A184" s="1">
         <v>45504</v>
       </c>
-      <c r="B184" t="n">
+      <c r="B184">
         <v>3511.25</v>
       </c>
     </row>
-    <row r="185">
-      <c r="A185" s="1" t="n">
+    <row r="185" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A185" s="1">
         <v>45505</v>
       </c>
-      <c r="B185" t="n">
+      <c r="B185">
         <v>2366.31</v>
       </c>
     </row>
-    <row r="186">
-      <c r="A186" s="1" t="n">
+    <row r="186" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A186" s="1">
         <v>45506</v>
       </c>
-      <c r="B186" t="n">
+      <c r="B186">
         <v>2204.92</v>
       </c>
     </row>
-    <row r="187">
-      <c r="A187" s="1" t="n">
+    <row r="187" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A187" s="1">
         <v>45508</v>
       </c>
-      <c r="B187" t="n">
+      <c r="B187">
         <v>3090.46</v>
       </c>
     </row>
-    <row r="188">
-      <c r="A188" s="1" t="n">
+    <row r="188" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A188" s="1">
         <v>45509</v>
       </c>
-      <c r="B188" t="n">
-        <v>2374.28</v>
-      </c>
-    </row>
-    <row r="189">
-      <c r="A189" s="1" t="n">
+      <c r="B188">
+        <v>2374.2800000000002</v>
+      </c>
+    </row>
+    <row r="189" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A189" s="1">
         <v>45511</v>
       </c>
-      <c r="B189" t="n">
+      <c r="B189">
         <v>1650.74</v>
       </c>
     </row>
-    <row r="190">
-      <c r="A190" s="1" t="n">
+    <row r="190" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A190" s="1">
         <v>45512</v>
       </c>
-      <c r="B190" t="n">
+      <c r="B190">
         <v>4185.62</v>
       </c>
     </row>
-    <row r="191">
-      <c r="A191" s="1" t="n">
+    <row r="191" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A191" s="1">
         <v>45513</v>
       </c>
-      <c r="B191" t="n">
+      <c r="B191">
         <v>3732.72</v>
       </c>
     </row>
-    <row r="192">
-      <c r="A192" s="1" t="n">
+    <row r="192" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A192" s="1">
         <v>45514</v>
       </c>
-      <c r="B192" t="n">
+      <c r="B192">
         <v>3661.73</v>
       </c>
     </row>
-    <row r="193">
-      <c r="A193" s="1" t="n">
+    <row r="193" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A193" s="1">
         <v>45515</v>
       </c>
-      <c r="B193" t="n">
+      <c r="B193">
         <v>2442</v>
       </c>
     </row>
-    <row r="194">
-      <c r="A194" s="1" t="n">
+    <row r="194" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A194" s="1">
         <v>45516</v>
       </c>
-      <c r="B194" t="n">
+      <c r="B194">
         <v>4529.25</v>
       </c>
     </row>
-    <row r="195">
-      <c r="A195" s="1" t="n">
+    <row r="195" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A195" s="1">
         <v>45517</v>
       </c>
-      <c r="B195" t="n">
+      <c r="B195">
         <v>2923.85</v>
       </c>
     </row>
-    <row r="196">
-      <c r="A196" s="1" t="n">
+    <row r="196" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A196" s="1">
         <v>45518</v>
       </c>
-      <c r="B196" t="n">
+      <c r="B196">
         <v>3091.22</v>
       </c>
     </row>
-    <row r="197">
-      <c r="A197" s="1" t="n">
+    <row r="197" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A197" s="1">
         <v>45519</v>
       </c>
-      <c r="B197" t="n">
+      <c r="B197">
         <v>4001.1</v>
       </c>
     </row>
-    <row r="198">
-      <c r="A198" s="1" t="n">
+    <row r="198" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A198" s="1">
         <v>45520</v>
       </c>
-      <c r="B198" t="n">
+      <c r="B198">
         <v>1899.36</v>
       </c>
     </row>
-    <row r="199">
-      <c r="A199" s="1" t="n">
+    <row r="199" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A199" s="1">
         <v>45521</v>
       </c>
-      <c r="B199" t="n">
+      <c r="B199">
         <v>4764.2</v>
       </c>
     </row>
-    <row r="200">
-      <c r="A200" s="1" t="n">
+    <row r="200" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A200" s="1">
         <v>45523</v>
       </c>
-      <c r="B200" t="n">
+      <c r="B200">
         <v>1726.39</v>
       </c>
     </row>
-    <row r="201">
-      <c r="A201" s="1" t="n">
+    <row r="201" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A201" s="1">
         <v>45524</v>
       </c>
-      <c r="B201" t="n">
+      <c r="B201">
         <v>3370.92</v>
       </c>
     </row>
-    <row r="202">
-      <c r="A202" s="1" t="n">
+    <row r="202" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A202" s="1">
         <v>45525</v>
       </c>
-      <c r="B202" t="n">
+      <c r="B202">
         <v>4571.32</v>
       </c>
     </row>
-    <row r="203">
-      <c r="A203" s="1" t="n">
+    <row r="203" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A203" s="1">
         <v>45526</v>
       </c>
-      <c r="B203" t="n">
+      <c r="B203">
         <v>3390.83</v>
       </c>
     </row>
-    <row r="204">
-      <c r="A204" s="1" t="n">
+    <row r="204" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A204" s="1">
         <v>45527</v>
       </c>
-      <c r="B204" t="n">
+      <c r="B204">
         <v>1557.68</v>
       </c>
     </row>
-    <row r="205">
-      <c r="A205" s="1" t="n">
+    <row r="205" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A205" s="1">
         <v>45528</v>
       </c>
-      <c r="B205" t="n">
+      <c r="B205">
         <v>4236.51</v>
       </c>
     </row>
-    <row r="206">
-      <c r="A206" s="1" t="n">
+    <row r="206" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A206" s="1">
         <v>45529</v>
       </c>
-      <c r="B206" t="n">
+      <c r="B206">
         <v>4531.37</v>
       </c>
     </row>
-    <row r="207">
-      <c r="A207" s="1" t="n">
+    <row r="207" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A207" s="1">
         <v>45530</v>
       </c>
-      <c r="B207" t="n">
+      <c r="B207">
         <v>2971.29</v>
       </c>
     </row>
-    <row r="208">
-      <c r="A208" s="1" t="n">
+    <row r="208" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A208" s="1">
         <v>45531</v>
       </c>
-      <c r="B208" t="n">
+      <c r="B208">
         <v>1975.6</v>
       </c>
     </row>
-    <row r="209">
-      <c r="A209" s="1" t="n">
+    <row r="209" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A209" s="1">
         <v>45532</v>
       </c>
-      <c r="B209" t="n">
-        <v>2158.99</v>
-      </c>
-    </row>
-    <row r="210">
-      <c r="A210" s="1" t="n">
+      <c r="B209">
+        <v>2158.9899999999998</v>
+      </c>
+    </row>
+    <row r="210" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A210" s="1">
         <v>45533</v>
       </c>
-      <c r="B210" t="n">
-        <v>2460.72</v>
-      </c>
-    </row>
-    <row r="211">
-      <c r="A211" s="1" t="n">
+      <c r="B210">
+        <v>2460.7199999999998</v>
+      </c>
+    </row>
+    <row r="211" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A211" s="1">
         <v>45536</v>
       </c>
-      <c r="B211" t="n">
+      <c r="B211">
         <v>3662.07</v>
       </c>
     </row>
-    <row r="212">
-      <c r="A212" s="1" t="n">
+    <row r="212" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A212" s="1">
         <v>45539</v>
       </c>
-      <c r="B212" t="n">
-        <v>4379.86</v>
-      </c>
-    </row>
-    <row r="213">
-      <c r="A213" s="1" t="n">
+      <c r="B212">
+        <v>4379.8599999999997</v>
+      </c>
+    </row>
+    <row r="213" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A213" s="1">
         <v>45542</v>
       </c>
-      <c r="B213" t="n">
+      <c r="B213">
         <v>4690.59</v>
       </c>
     </row>
-    <row r="214">
-      <c r="A214" s="1" t="n">
+    <row r="214" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A214" s="1">
         <v>45543</v>
       </c>
-      <c r="B214" t="n">
+      <c r="B214">
         <v>2961.1</v>
       </c>
     </row>
-    <row r="215">
-      <c r="A215" s="1" t="n">
+    <row r="215" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A215" s="1">
         <v>45544</v>
       </c>
-      <c r="B215" t="n">
+      <c r="B215">
         <v>1861.56</v>
       </c>
     </row>
-    <row r="216">
-      <c r="A216" s="1" t="n">
+    <row r="216" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A216" s="1">
         <v>45545</v>
       </c>
-      <c r="B216" t="n">
-        <v>4263.27</v>
-      </c>
-    </row>
-    <row r="217">
-      <c r="A217" s="1" t="n">
+      <c r="B216">
+        <v>4263.2700000000004</v>
+      </c>
+    </row>
+    <row r="217" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A217" s="1">
         <v>45547</v>
       </c>
-      <c r="B217" t="n">
+      <c r="B217">
         <v>2495.6</v>
       </c>
     </row>
-    <row r="218">
-      <c r="A218" s="1" t="n">
+    <row r="218" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A218" s="1">
         <v>45548</v>
       </c>
-      <c r="B218" t="n">
+      <c r="B218">
         <v>3387.43</v>
       </c>
     </row>
-    <row r="219">
-      <c r="A219" s="1" t="n">
+    <row r="219" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A219" s="1">
         <v>45549</v>
       </c>
-      <c r="B219" t="n">
+      <c r="B219">
         <v>3239.56</v>
       </c>
     </row>
-    <row r="220">
-      <c r="A220" s="1" t="n">
+    <row r="220" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A220" s="1">
         <v>45550</v>
       </c>
-      <c r="B220" t="n">
+      <c r="B220">
         <v>2256.41</v>
       </c>
     </row>
-    <row r="221">
-      <c r="A221" s="1" t="n">
+    <row r="221" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A221" s="1">
         <v>45551</v>
       </c>
-      <c r="B221" t="n">
+      <c r="B221">
         <v>3720.65</v>
       </c>
     </row>
-    <row r="222">
-      <c r="A222" s="1" t="n">
+    <row r="222" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A222" s="1">
         <v>45553</v>
       </c>
-      <c r="B222" t="n">
+      <c r="B222">
         <v>4929.07</v>
       </c>
     </row>
-    <row r="223">
-      <c r="A223" s="1" t="n">
+    <row r="223" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A223" s="1">
         <v>45554</v>
       </c>
-      <c r="B223" t="n">
+      <c r="B223">
         <v>2317.08</v>
       </c>
     </row>
-    <row r="224">
-      <c r="A224" s="1" t="n">
+    <row r="224" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A224" s="1">
         <v>45556</v>
       </c>
-      <c r="B224" t="n">
+      <c r="B224">
         <v>3658.24</v>
       </c>
     </row>
-    <row r="225">
-      <c r="A225" s="1" t="n">
+    <row r="225" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A225" s="1">
         <v>45557</v>
       </c>
-      <c r="B225" t="n">
+      <c r="B225">
         <v>3552.08</v>
       </c>
     </row>
-    <row r="226">
-      <c r="A226" s="1" t="n">
+    <row r="226" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A226" s="1">
         <v>45558</v>
       </c>
-      <c r="B226" t="n">
+      <c r="B226">
         <v>4241.17</v>
       </c>
     </row>
-    <row r="227">
-      <c r="A227" s="1" t="n">
+    <row r="227" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A227" s="1">
         <v>45560</v>
       </c>
-      <c r="B227" t="n">
-        <v>4198.35</v>
-      </c>
-    </row>
-    <row r="228">
-      <c r="A228" s="1" t="n">
+      <c r="B227">
+        <v>4198.3500000000004</v>
+      </c>
+    </row>
+    <row r="228" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A228" s="1">
         <v>45561</v>
       </c>
-      <c r="B228" t="n">
+      <c r="B228">
         <v>2188.9</v>
       </c>
     </row>
-    <row r="229">
-      <c r="A229" s="1" t="n">
+    <row r="229" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A229" s="1">
         <v>45562</v>
       </c>
-      <c r="B229" t="n">
+      <c r="B229">
         <v>4713.91</v>
       </c>
     </row>
-    <row r="230">
-      <c r="A230" s="1" t="n">
+    <row r="230" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A230" s="1">
         <v>45564</v>
       </c>
-      <c r="B230" t="n">
+      <c r="B230">
         <v>1918.39</v>
       </c>
     </row>
-    <row r="231">
-      <c r="A231" s="1" t="n">
+    <row r="231" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A231" s="1">
         <v>45565</v>
       </c>
-      <c r="B231" t="n">
+      <c r="B231">
         <v>1561.85</v>
       </c>
     </row>
-    <row r="232">
-      <c r="A232" s="1" t="n">
+    <row r="232" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A232" s="1">
         <v>45566</v>
       </c>
-      <c r="B232" t="n">
+      <c r="B232">
         <v>3659.99</v>
       </c>
     </row>
-    <row r="233">
-      <c r="A233" s="1" t="n">
+    <row r="233" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A233" s="1">
         <v>45567</v>
       </c>
-      <c r="B233" t="n">
+      <c r="B233">
         <v>3836.77</v>
       </c>
     </row>
-    <row r="234">
-      <c r="A234" s="1" t="n">
+    <row r="234" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A234" s="1">
         <v>45569</v>
       </c>
-      <c r="B234" t="n">
+      <c r="B234">
         <v>3503.27</v>
       </c>
     </row>
-    <row r="235">
-      <c r="A235" s="1" t="n">
+    <row r="235" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A235" s="1">
         <v>45571</v>
       </c>
-      <c r="B235" t="n">
+      <c r="B235">
         <v>3667.2</v>
       </c>
     </row>
-    <row r="236">
-      <c r="A236" s="1" t="n">
+    <row r="236" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A236" s="1">
         <v>45572</v>
       </c>
-      <c r="B236" t="n">
+      <c r="B236">
         <v>3453.55</v>
       </c>
     </row>
-    <row r="237">
-      <c r="A237" s="1" t="n">
+    <row r="237" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A237" s="1">
         <v>45573</v>
       </c>
-      <c r="B237" t="n">
+      <c r="B237">
         <v>3997.64</v>
       </c>
     </row>
-    <row r="238">
-      <c r="A238" s="1" t="n">
+    <row r="238" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A238" s="1">
         <v>45574</v>
       </c>
-      <c r="B238" t="n">
+      <c r="B238">
         <v>3863.46</v>
       </c>
     </row>
-    <row r="239">
-      <c r="A239" s="1" t="n">
+    <row r="239" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A239" s="1">
         <v>45576</v>
       </c>
-      <c r="B239" t="n">
+      <c r="B239">
         <v>4090.93</v>
       </c>
     </row>
-    <row r="240">
-      <c r="A240" s="1" t="n">
+    <row r="240" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A240" s="1">
         <v>45577</v>
       </c>
-      <c r="B240" t="n">
+      <c r="B240">
         <v>2255.63</v>
       </c>
     </row>
-    <row r="241">
-      <c r="A241" s="1" t="n">
+    <row r="241" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A241" s="1">
         <v>45578</v>
       </c>
-      <c r="B241" t="n">
+      <c r="B241">
         <v>3771.71</v>
       </c>
     </row>
-    <row r="242">
-      <c r="A242" s="1" t="n">
+    <row r="242" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A242" s="1">
         <v>45580</v>
       </c>
-      <c r="B242" t="n">
-        <v>4368.73</v>
-      </c>
-    </row>
-    <row r="243">
-      <c r="A243" s="1" t="n">
+      <c r="B242">
+        <v>4368.7299999999996</v>
+      </c>
+    </row>
+    <row r="243" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A243" s="1">
         <v>45582</v>
       </c>
-      <c r="B243" t="n">
+      <c r="B243">
         <v>2952.8</v>
       </c>
     </row>
-    <row r="244">
-      <c r="A244" s="1" t="n">
+    <row r="244" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A244" s="1">
         <v>45584</v>
       </c>
-      <c r="B244" t="n">
+      <c r="B244">
         <v>3657.3</v>
       </c>
     </row>
-    <row r="245">
-      <c r="A245" s="1" t="n">
+    <row r="245" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A245" s="1">
         <v>45585</v>
       </c>
-      <c r="B245" t="n">
+      <c r="B245">
         <v>4642.57</v>
       </c>
     </row>
-    <row r="246">
-      <c r="A246" s="1" t="n">
+    <row r="246" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A246" s="1">
         <v>45587</v>
       </c>
-      <c r="B246" t="n">
+      <c r="B246">
         <v>3313.05</v>
       </c>
     </row>
-    <row r="247">
-      <c r="A247" s="1" t="n">
+    <row r="247" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A247" s="1">
         <v>45588</v>
       </c>
-      <c r="B247" t="n">
+      <c r="B247">
         <v>3855.38</v>
       </c>
     </row>
-    <row r="248">
-      <c r="A248" s="1" t="n">
+    <row r="248" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A248" s="1">
         <v>45589</v>
       </c>
-      <c r="B248" t="n">
+      <c r="B248">
         <v>3533.35</v>
       </c>
     </row>
-    <row r="249">
-      <c r="A249" s="1" t="n">
+    <row r="249" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A249" s="1">
         <v>45590</v>
       </c>
-      <c r="B249" t="n">
+      <c r="B249">
         <v>2054</v>
       </c>
     </row>
-    <row r="250">
-      <c r="A250" s="1" t="n">
+    <row r="250" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A250" s="1">
         <v>45591</v>
       </c>
-      <c r="B250" t="n">
+      <c r="B250">
         <v>4317.34</v>
       </c>
     </row>
-    <row r="251">
-      <c r="A251" s="1" t="n">
+    <row r="251" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A251" s="1">
         <v>45592</v>
       </c>
-      <c r="B251" t="n">
-        <v>4720.1</v>
-      </c>
-    </row>
-    <row r="252">
-      <c r="A252" s="1" t="n">
+      <c r="B251">
+        <v>4720.1000000000004</v>
+      </c>
+    </row>
+    <row r="252" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A252" s="1">
         <v>45593</v>
       </c>
-      <c r="B252" t="n">
+      <c r="B252">
         <v>3196.09</v>
       </c>
     </row>
-    <row r="253">
-      <c r="A253" s="1" t="n">
+    <row r="253" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A253" s="1">
         <v>45595</v>
       </c>
-      <c r="B253" t="n">
+      <c r="B253">
         <v>3165.38</v>
       </c>
     </row>
-    <row r="254">
-      <c r="A254" s="1" t="n">
+    <row r="254" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A254" s="1">
         <v>45596</v>
       </c>
-      <c r="B254" t="n">
+      <c r="B254">
         <v>1781.26</v>
       </c>
     </row>
-    <row r="255">
-      <c r="A255" s="1" t="n">
+    <row r="255" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A255" s="1">
         <v>45597</v>
       </c>
-      <c r="B255" t="n">
+      <c r="B255">
         <v>2791.76</v>
       </c>
     </row>
-    <row r="256">
-      <c r="A256" s="1" t="n">
+    <row r="256" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A256" s="1">
         <v>45598</v>
       </c>
-      <c r="B256" t="n">
+      <c r="B256">
         <v>4623.78</v>
       </c>
     </row>
-    <row r="257">
-      <c r="A257" s="1" t="n">
+    <row r="257" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A257" s="1">
         <v>45599</v>
       </c>
-      <c r="B257" t="n">
+      <c r="B257">
         <v>3731.55</v>
       </c>
     </row>
-    <row r="258">
-      <c r="A258" s="1" t="n">
+    <row r="258" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A258" s="1">
         <v>45600</v>
       </c>
-      <c r="B258" t="n">
+      <c r="B258">
         <v>3942.11</v>
       </c>
     </row>
-    <row r="259">
-      <c r="A259" s="1" t="n">
+    <row r="259" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A259" s="1">
         <v>45601</v>
       </c>
-      <c r="B259" t="n">
+      <c r="B259">
         <v>4186.3</v>
       </c>
     </row>
-    <row r="260">
-      <c r="A260" s="1" t="n">
+    <row r="260" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A260" s="1">
         <v>45602</v>
       </c>
-      <c r="B260" t="n">
+      <c r="B260">
         <v>4342.2</v>
       </c>
     </row>
-    <row r="261">
-      <c r="A261" s="1" t="n">
+    <row r="261" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A261" s="1">
         <v>45603</v>
       </c>
-      <c r="B261" t="n">
+      <c r="B261">
         <v>3636.17</v>
       </c>
     </row>
-    <row r="262">
-      <c r="A262" s="1" t="n">
+    <row r="262" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A262" s="1">
         <v>45605</v>
       </c>
-      <c r="B262" t="n">
+      <c r="B262">
         <v>4645.49</v>
       </c>
     </row>
-    <row r="263">
-      <c r="A263" s="1" t="n">
+    <row r="263" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A263" s="1">
         <v>45607</v>
       </c>
-      <c r="B263" t="n">
+      <c r="B263">
         <v>3049.42</v>
       </c>
     </row>
-    <row r="264">
-      <c r="A264" s="1" t="n">
+    <row r="264" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A264" s="1">
         <v>45609</v>
       </c>
-      <c r="B264" t="n">
+      <c r="B264">
         <v>3173.98</v>
       </c>
     </row>
-    <row r="265">
-      <c r="A265" s="1" t="n">
+    <row r="265" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A265" s="1">
         <v>45610</v>
       </c>
-      <c r="B265" t="n">
+      <c r="B265">
         <v>3606.59</v>
       </c>
     </row>
-    <row r="266">
-      <c r="A266" s="1" t="n">
+    <row r="266" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A266" s="1">
         <v>45611</v>
       </c>
-      <c r="B266" t="n">
-        <v>2504.22</v>
-      </c>
-    </row>
-    <row r="267">
-      <c r="A267" s="1" t="n">
+      <c r="B266">
+        <v>2504.2199999999998</v>
+      </c>
+    </row>
+    <row r="267" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A267" s="1">
         <v>45613</v>
       </c>
-      <c r="B267" t="n">
+      <c r="B267">
         <v>4291.74</v>
       </c>
     </row>
-    <row r="268">
-      <c r="A268" s="1" t="n">
+    <row r="268" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A268" s="1">
         <v>45614</v>
       </c>
-      <c r="B268" t="n">
+      <c r="B268">
         <v>2931.87</v>
       </c>
     </row>
-    <row r="269">
-      <c r="A269" s="1" t="n">
+    <row r="269" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A269" s="1">
         <v>45615</v>
       </c>
-      <c r="B269" t="n">
-        <v>4817.4</v>
-      </c>
-    </row>
-    <row r="270">
-      <c r="A270" s="1" t="n">
+      <c r="B269">
+        <v>4817.3999999999996</v>
+      </c>
+    </row>
+    <row r="270" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A270" s="1">
         <v>45616</v>
       </c>
-      <c r="B270" t="n">
+      <c r="B270">
         <v>2819.38</v>
       </c>
     </row>
-    <row r="271">
-      <c r="A271" s="1" t="n">
+    <row r="271" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A271" s="1">
         <v>45617</v>
       </c>
-      <c r="B271" t="n">
+      <c r="B271">
         <v>4103.91</v>
       </c>
     </row>
-    <row r="272">
-      <c r="A272" s="1" t="n">
+    <row r="272" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A272" s="1">
         <v>45618</v>
       </c>
-      <c r="B272" t="n">
-        <v>4202.85</v>
-      </c>
-    </row>
-    <row r="273">
-      <c r="A273" s="1" t="n">
+      <c r="B272">
+        <v>4202.8500000000004</v>
+      </c>
+    </row>
+    <row r="273" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A273" s="1">
         <v>45619</v>
       </c>
-      <c r="B273" t="n">
+      <c r="B273">
         <v>1565.02</v>
       </c>
     </row>
-    <row r="274">
-      <c r="A274" s="1" t="n">
+    <row r="274" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A274" s="1">
         <v>45620</v>
       </c>
-      <c r="B274" t="n">
+      <c r="B274">
         <v>3529.66</v>
       </c>
     </row>
-    <row r="275">
-      <c r="A275" s="1" t="n">
+    <row r="275" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A275" s="1">
         <v>45621</v>
       </c>
-      <c r="B275" t="n">
+      <c r="B275">
         <v>2797.95</v>
       </c>
     </row>
-    <row r="276">
-      <c r="A276" s="1" t="n">
+    <row r="276" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A276" s="1">
         <v>45622</v>
       </c>
-      <c r="B276" t="n">
-        <v>2276.2</v>
-      </c>
-    </row>
-    <row r="277">
-      <c r="A277" s="1" t="n">
+      <c r="B276">
+        <v>2276.1999999999998</v>
+      </c>
+    </row>
+    <row r="277" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A277" s="1">
         <v>45623</v>
       </c>
-      <c r="B277" t="n">
+      <c r="B277">
         <v>2918.72</v>
       </c>
     </row>
-    <row r="278">
-      <c r="A278" s="1" t="n">
+    <row r="278" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A278" s="1">
         <v>45624</v>
       </c>
-      <c r="B278" t="n">
+      <c r="B278">
         <v>1693.27</v>
       </c>
     </row>
-    <row r="279">
-      <c r="A279" s="1" t="n">
+    <row r="279" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A279" s="1">
         <v>45625</v>
       </c>
-      <c r="B279" t="n">
+      <c r="B279">
         <v>3612.07</v>
       </c>
     </row>
-    <row r="280">
-      <c r="A280" s="1" t="n">
+    <row r="280" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A280" s="1">
         <v>45626</v>
       </c>
-      <c r="B280" t="n">
+      <c r="B280">
         <v>4566.53</v>
       </c>
     </row>
-    <row r="281">
-      <c r="A281" s="1" t="n">
+    <row r="281" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A281" s="1">
         <v>45628</v>
       </c>
-      <c r="B281" t="n">
-        <v>4367.11</v>
-      </c>
-    </row>
-    <row r="282">
-      <c r="A282" s="1" t="n">
+      <c r="B281">
+        <v>4367.1099999999997</v>
+      </c>
+    </row>
+    <row r="282" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A282" s="1">
         <v>45629</v>
       </c>
-      <c r="B282" t="n">
+      <c r="B282">
         <v>4517.84</v>
       </c>
     </row>
-    <row r="283">
-      <c r="A283" s="1" t="n">
+    <row r="283" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A283" s="1">
         <v>45631</v>
       </c>
-      <c r="B283" t="n">
+      <c r="B283">
         <v>4501.42</v>
       </c>
     </row>
-    <row r="284">
-      <c r="A284" s="1" t="n">
+    <row r="284" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A284" s="1">
         <v>45632</v>
       </c>
-      <c r="B284" t="n">
+      <c r="B284">
         <v>1796.84</v>
       </c>
     </row>
-    <row r="285">
-      <c r="A285" s="1" t="n">
+    <row r="285" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A285" s="1">
         <v>45633</v>
       </c>
-      <c r="B285" t="n">
+      <c r="B285">
         <v>3194.68</v>
       </c>
     </row>
-    <row r="286">
-      <c r="A286" s="1" t="n">
+    <row r="286" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A286" s="1">
         <v>45634</v>
       </c>
-      <c r="B286" t="n">
+      <c r="B286">
         <v>3334.03</v>
       </c>
     </row>
-    <row r="287">
-      <c r="A287" s="1" t="n">
+    <row r="287" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A287" s="1">
         <v>45636</v>
       </c>
-      <c r="B287" t="n">
+      <c r="B287">
         <v>1748.97</v>
       </c>
     </row>
-    <row r="288">
-      <c r="A288" s="1" t="n">
+    <row r="288" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A288" s="1">
         <v>45638</v>
       </c>
-      <c r="B288" t="n">
-        <v>4381.11</v>
-      </c>
-    </row>
-    <row r="289">
-      <c r="A289" s="1" t="n">
+      <c r="B288">
+        <v>4381.1099999999997</v>
+      </c>
+    </row>
+    <row r="289" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A289" s="1">
         <v>45639</v>
       </c>
-      <c r="B289" t="n">
+      <c r="B289">
         <v>3911.03</v>
       </c>
     </row>
-    <row r="290">
-      <c r="A290" s="1" t="n">
+    <row r="290" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A290" s="1">
         <v>45640</v>
       </c>
-      <c r="B290" t="n">
+      <c r="B290">
         <v>2332.54</v>
       </c>
     </row>
-    <row r="291">
-      <c r="A291" s="1" t="n">
+    <row r="291" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A291" s="1">
         <v>45641</v>
       </c>
-      <c r="B291" t="n">
+      <c r="B291">
         <v>2181.4</v>
       </c>
     </row>
-    <row r="292">
-      <c r="A292" s="1" t="n">
+    <row r="292" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A292" s="1">
         <v>45643</v>
       </c>
-      <c r="B292" t="n">
+      <c r="B292">
         <v>2871.11</v>
       </c>
     </row>
-    <row r="293">
-      <c r="A293" s="1" t="n">
+    <row r="293" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A293" s="1">
         <v>45646</v>
       </c>
-      <c r="B293" t="n">
-        <v>4892.6</v>
-      </c>
-    </row>
-    <row r="294">
-      <c r="A294" s="1" t="n">
+      <c r="B293">
+        <v>4892.6000000000004</v>
+      </c>
+    </row>
+    <row r="294" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A294" s="1">
         <v>45647</v>
       </c>
-      <c r="B294" t="n">
+      <c r="B294">
         <v>3389.54</v>
       </c>
     </row>
-    <row r="295">
-      <c r="A295" s="1" t="n">
+    <row r="295" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A295" s="1">
         <v>45649</v>
       </c>
-      <c r="B295" t="n">
+      <c r="B295">
         <v>4729.47</v>
       </c>
     </row>
-    <row r="296">
-      <c r="A296" s="1" t="n">
+    <row r="296" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A296" s="1">
         <v>45650</v>
       </c>
-      <c r="B296" t="n">
-        <v>4977.64</v>
-      </c>
-    </row>
-    <row r="297">
-      <c r="A297" s="1" t="n">
+      <c r="B296">
+        <v>4977.6400000000003</v>
+      </c>
+    </row>
+    <row r="297" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A297" s="1">
         <v>45651</v>
       </c>
-      <c r="B297" t="n">
+      <c r="B297">
         <v>3177.18</v>
       </c>
     </row>
-    <row r="298">
-      <c r="A298" s="1" t="n">
+    <row r="298" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A298" s="1">
         <v>45654</v>
       </c>
-      <c r="B298" t="n">
+      <c r="B298">
         <v>2531.02</v>
       </c>
     </row>
-    <row r="299">
-      <c r="A299" s="1" t="n">
+    <row r="299" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A299" s="1">
         <v>45655</v>
       </c>
-      <c r="B299" t="n">
+      <c r="B299">
         <v>4137.24</v>
       </c>
     </row>
-    <row r="300">
-      <c r="A300" s="1" t="n">
+    <row r="300" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A300" s="1">
         <v>45657</v>
       </c>
-      <c r="B300" t="n">
-        <v>2417.03</v>
+      <c r="B300">
+        <v>2417.0300000000002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>